<commit_message>
sync dados_graficos 15/05/2026  9:26:13,38
</commit_message>
<xml_diff>
--- a/dados_graficos/dados_graficos.xlsx
+++ b/dados_graficos/dados_graficos.xlsx
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>726</v>
+        <v>709</v>
       </c>
     </row>
     <row r="3">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>14139</v>
+        <v>14453</v>
       </c>
     </row>
     <row r="7">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>3761</v>
+        <v>3046</v>
       </c>
     </row>
     <row r="8">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>421</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>8408</v>
+        <v>8704</v>
       </c>
     </row>
     <row r="10">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>483</v>
+        <v>457</v>
       </c>
     </row>
     <row r="11"/>

</xml_diff>

<commit_message>
sync dados_graficos 18/05/2026 10:30:16,54
</commit_message>
<xml_diff>
--- a/dados_graficos/dados_graficos.xlsx
+++ b/dados_graficos/dados_graficos.xlsx
@@ -3,20 +3,20 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,39 +32,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -87,41 +64,15 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,13 +438,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="23" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="31.140625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="9.140625" customWidth="1" style="3" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -501,119 +447,118 @@
           <t>Funcao</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>col_2</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Erros</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>checar_alunos_total</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
-        <v>181175</v>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="B2" t="n">
+        <v>181193</v>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>CPF inválido/em branco</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n">
-        <v>709</v>
+      <c r="D2" t="n">
+        <v>690</v>
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Matrícula duplicada</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Deficiência sem descrição</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" t="n">
         <v>5</v>
       </c>
-      <c r="H4" s="8" t="n"/>
     </row>
     <row r="5">
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Descrição de deficiência indevida</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
-        <v>69</v>
+      <c r="D5" t="n">
+        <v>71</v>
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>dt_matricula alterada</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
-        <v>14453</v>
+      <c r="D6" t="n">
+        <v>14501</v>
       </c>
     </row>
     <row r="7">
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Matrícula retroativa</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>3046</v>
+      <c r="D7" t="n">
+        <v>3054</v>
       </c>
     </row>
     <row r="8">
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mudança de id_aluno</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
-        <v>284</v>
+      <c r="D8" t="n">
+        <v>285</v>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Frequência io-iô</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
-        <v>8704</v>
+      <c r="D9" t="n">
+        <v>8746</v>
       </c>
     </row>
     <row r="10">
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Sem_autodeclaracao_racial</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n">
-        <v>457</v>
+      <c r="D10" t="n">
+        <v>455</v>
       </c>
     </row>
     <row r="11"/>
@@ -628,6 +573,5 @@
     <row r="20"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
sync dados_graficos 19/05/2026  8:03:55,89
</commit_message>
<xml_diff>
--- a/dados_graficos/dados_graficos.xlsx
+++ b/dados_graficos/dados_graficos.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>181193</v>
+        <v>181023</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>690</v>
+        <v>685</v>
       </c>
     </row>
     <row r="3">
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14501</v>
+        <v>14645</v>
       </c>
     </row>
     <row r="7">
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3054</v>
+        <v>3056</v>
       </c>
     </row>
     <row r="8">
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="9">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8746</v>
+        <v>8844</v>
       </c>
     </row>
     <row r="10">
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>455</v>
+        <v>446</v>
       </c>
     </row>
     <row r="11"/>

</xml_diff>

<commit_message>
sync dados_graficos 03/06/2026  8:53:04,69
</commit_message>
<xml_diff>
--- a/dados_graficos/dados_graficos.xlsx
+++ b/dados_graficos/dados_graficos.xlsx
@@ -1,33 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -41,7 +33,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,30 +41,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,20 +412,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="B1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.7109375" customWidth="1" min="2" max="2"/>
+    <col width="26.85546875" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Funcao</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Resultado</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
           <t>col_2</t>
@@ -464,13 +433,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>checar_alunos_total</t>
-        </is>
-      </c>
       <c r="B2" t="n">
-        <v>181023</v>
+        <v>182461</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -478,7 +442,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>685</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3">
@@ -498,7 +462,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -508,7 +472,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6">
@@ -518,7 +482,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14645</v>
+        <v>15774</v>
       </c>
     </row>
     <row r="7">
@@ -528,7 +492,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3056</v>
+        <v>4019</v>
       </c>
     </row>
     <row r="8">
@@ -538,7 +502,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>286</v>
+        <v>479</v>
       </c>
     </row>
     <row r="9">
@@ -548,7 +512,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8844</v>
+        <v>9846</v>
       </c>
     </row>
     <row r="10">
@@ -558,10 +522,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="11"/>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Última aparição anterior a hoje</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4808</v>
+      </c>
+    </row>
     <row r="12"/>
     <row r="13"/>
     <row r="14"/>
@@ -572,6 +545,6 @@
     <row r="19"/>
     <row r="20"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>